<commit_message>
Set loan start to Jun 2026 (real start) in Excel + local web app
- Excel start date -> Jun 2026; recalc-verified (math unchanged, dates corrected)
- Web app default start -> 2026-06 for the local pre-filled build; 14 tests pass
- Public GitHub Pages deploy uses the generic build (no personal data)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Home-Loan-Prepayment-Planner.xlsx
+++ b/Home-Loan-Prepayment-Planner.xlsx
@@ -721,10 +721,10 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>45658</v>
+        <v>46174</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>45658</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Correct Loan A to real figures from HDFC statement + pre-EMI
- Loan A: Rs 35,00,000 @ 7.25%, 180mo (was placeholder 30L@7.5%) per HDFC
  provisional statement a/c 704937787; under-construction, full EMI from Jul 2026
- Pre-EMI interest Rs 17,877 recorded (one-time sunk cost; does not change savings)
- EMI now Rs 31,951; baseline interest Rs 22,50,921 (Rs 22,68,798 incl pre-EMI)
- Excel + verifier + web defaults + smoke tests updated; 14 web tests + Excel recalc pass

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Home-Loan-Prepayment-Planner.xlsx
+++ b/Home-Loan-Prepayment-Planner.xlsx
@@ -648,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -682,7 +682,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>3000000</v>
+        <v>3500000</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>5000000</v>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>7.5</v>
+        <v>7.25</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>7.5</v>
@@ -717,14 +717,14 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>EMI start date</t>
+          <t>Full-EMI start date</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="7">
@@ -755,6 +755,19 @@
       <c r="C8" s="8">
         <f>C4/100/12</f>
         <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Pre-EMI interest (one-time)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>17877</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -22608,7 +22621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -22834,6 +22847,51 @@
       </c>
       <c r="B16" s="22">
         <f>IF(Inputs!B4&gt;Inputs!C4,"Loan A (higher rate)",IF(Inputs!C4&gt;Inputs!B4,"Loan B (higher rate)",IF(Inputs!B3&gt;=Inputs!C3,"Loan B (larger balance saves more)","Loan A (larger balance saves more)")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Note: pre-EMI is interest-only and does not change months/interest saved above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Pre-EMI interest (one-time)</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>Inputs!B9</f>
+        <v/>
+      </c>
+      <c r="C18" s="15">
+        <f>Inputs!C9</f>
+        <v/>
+      </c>
+      <c r="D18" s="15">
+        <f>B18+C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Total interest incl. pre-EMI (plan)</t>
+        </is>
+      </c>
+      <c r="B19" s="15">
+        <f>B7+B18</f>
+        <v/>
+      </c>
+      <c r="C19" s="15">
+        <f>C7+C18</f>
+        <v/>
+      </c>
+      <c r="D19" s="15">
+        <f>B19+C19</f>
         <v/>
       </c>
     </row>

</xml_diff>